<commit_message>
refactor: tighten public api surface
</commit_message>
<xml_diff>
--- a/test/res/typedef.xlsx
+++ b/test/res/typedef.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypes/Desktop/Github/xlsx-exporter/test/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68711C61-A5E7-974F-8FBB-C3AB25D5F8DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203FE284-D992-4D47-A4E1-C7F5D59A5BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1328,13 +1328,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
-<customStorage xmlns="https://web.wps.cn/et/2018/main">
-  <book/>
-  <sheets/>
-</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1730,7 +1723,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>29</v>
@@ -1842,7 +1835,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Support tuple typenames in generated outputs
</commit_message>
<xml_diff>
--- a/test/res/typedef.xlsx
+++ b/test/res/typedef.xlsx
@@ -2108,7 +2108,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A814D64C-E2BB-9F48-8DDA-58BFAA61AAAE}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="14.375" bestFit="1" customWidth="1"/>
@@ -2128,6 +2128,11 @@
       <c r="D1" s="11" t="s">
         <v>2</v>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
     </row>
     <row r="2" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
@@ -2142,6 +2147,11 @@
       <c r="D2" s="11" t="s">
         <v>32</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>[float, int][]?</t>
+        </is>
+      </c>
     </row>
     <row r="3" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
@@ -2152,6 +2162,11 @@
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="4" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
@@ -2166,6 +2181,11 @@
       <c r="D4" s="11" t="s">
         <v>3</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="5" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
@@ -2180,6 +2200,11 @@
       <c r="D5" s="14" t="s">
         <v>10</v>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>数据</t>
+        </is>
+      </c>
     </row>
     <row r="6" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A6" s="15">
@@ -2194,6 +2219,11 @@
       <c r="D6" s="18" t="s">
         <v>53</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>[[1.2,3], [1.55, 4]]</t>
+        </is>
+      </c>
     </row>
     <row r="7" spans="1:4" s="12" customFormat="1" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A7" s="15">
@@ -2207,6 +2237,11 @@
       </c>
       <c r="D7" s="19" t="s">
         <v>43</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>